<commit_message>
Met a jour le fichier de contribution par rubrique
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Maurice+ Contribution par rubrique.xlsx
+++ b/Maurice+ Contribution par rubrique.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Desktop\EXPAT\MAURICE APP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE3DC8A5-AA08-4269-A8F9-2850F834DBBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93625179-E6FC-4D6F-97A7-8261B88C438B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="12" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="1" r:id="rId1"/>
@@ -103,12 +103,25 @@
     <sheet name="EVT_Culturels" sheetId="86" r:id="rId88"/>
     <sheet name="EVT_Business" sheetId="87" r:id="rId89"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8455" uniqueCount="6521">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8458" uniqueCount="6524">
   <si>
     <t>Maurice+ — Contribution par rubrique</t>
   </si>
@@ -19682,6 +19695,15 @@
   </si>
   <si>
     <t>à mettre dans viewpoint</t>
+  </si>
+  <si>
+    <t>Demande en cours pour en rajouter (centre?!!)</t>
+  </si>
+  <si>
+    <t>Qu'est ce que le crayon et nom associé sur les fiches?</t>
+  </si>
+  <si>
+    <t>à compléter avec photo et court descriptif des randos</t>
   </si>
 </sst>
 </file>
@@ -19765,7 +19787,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -19782,6 +19804,12 @@
         <fgColor rgb="FFFFF9DB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -19796,7 +19824,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -19816,6 +19844,7 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -46108,7 +46137,7 @@
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="5" width="50" customWidth="1"/>
+    <col min="5" max="5" width="53.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
@@ -46119,6 +46148,11 @@
       <c r="C1" s="16"/>
       <c r="D1" s="16"/>
       <c r="E1" s="16"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>6521</v>
+      </c>
     </row>
     <row r="3" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -53825,6 +53859,11 @@
       <c r="C1" s="16"/>
       <c r="D1" s="16"/>
       <c r="E1" s="16"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>6522</v>
+      </c>
     </row>
     <row r="3" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -58834,7 +58873,7 @@
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="17" t="s">
         <v>6515</v>
       </c>
     </row>
@@ -59962,6 +60001,11 @@
       <c r="D1" s="16"/>
       <c r="E1" s="16"/>
     </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>6523</v>
+      </c>
+    </row>
     <row r="3" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>185</v>

</xml_diff>

<commit_message>
Cree la sous-rubrique Gym & fitness et reclasse les clubs sportifs, applique les corrections notees dans le fichier de contribution
- Nouvelle sous-rubrique "Gym & fitness" (famille Sports) : ~94 clubs de gym/fitness/crossfit deplaces ou tagges, complexes-sportifs recentre sur les equipements multisports
- Tennis/padel regroupes sous "Tennis & padel", PadelShop.mu vers Shopping
- Suppression de 3 doublons (Tennis Nord, Heritage Awali Golf and Spa Resort, Le Chateau de Bel Ombre)
- Wapalapam Island Eatery recategorise vers Activites/Malls
- Le Fangourin passe en coup de coeur (teste par l'utilisatrice)
- Descriptions originales ajoutees pour 5 sentiers de randonnee + nouvelle fiche Boucle courte des 7 Cascades
- Nouvelle fiche AD Events (Ecole du Nord), recherchee sur le web

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Maurice+ Contribution par rubrique.xlsx
+++ b/Maurice+ Contribution par rubrique.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Desktop\EXPAT\MAURICE APP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{060BE661-8AA4-4AC0-8B2D-1E551F4BF441}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF30AAD9-4164-4C56-981C-A8993C63404E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="13" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="1" r:id="rId1"/>
@@ -118,12 +118,16 @@
     <sheet name="EVT_Culturels" sheetId="103" r:id="rId103"/>
     <sheet name="EVT_Business" sheetId="104" r:id="rId104"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'ACT_Complexes sportifs'!$A$3:$E$179</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'ACT_Randonnée &amp; trail'!$A$3:$E$3</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10018" uniqueCount="7473">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10135" uniqueCount="7491">
   <si>
     <t>Maurice+ — Contribution par rubrique</t>
   </si>
@@ -22542,13 +22546,94 @@
   </si>
   <si>
     <t>Safari de 2h en 4*4. Note: vérifier qu ecelui ci est bien aussi dans réserves naturelels</t>
+  </si>
+  <si>
+    <t>à supprimer (doublon avec Vallée Adventaure)</t>
+  </si>
+  <si>
+    <t>à mettre dans activités enfants et famille</t>
+  </si>
+  <si>
+    <t>à mettre dans randonnée-trail</t>
+  </si>
+  <si>
+    <t>à supprimer doublon avec LSC</t>
+  </si>
+  <si>
+    <t>à déplacer dans shooping - magasins sport</t>
+  </si>
+  <si>
+    <t>à déplacer dans padel-tennis</t>
+  </si>
+  <si>
+    <t>à déplacer dans gym/fitness</t>
+  </si>
+  <si>
+    <t>à déplacer dans gym-fitness</t>
+  </si>
+  <si>
+    <t>compléter: 4,8km 500mD+. Attention aux moustqiues. Faire une synthèse plus courte de: Cet itinéraire est une entreprise aventureuse qui commence par une randonnée difficile à travers les champs de canne à sucre avant d'escalader l'épine dorsale de la montagne. Attendez-vous à un défi physique ; le sentier est accidenté, escarpé et souvent envahi par la végétation, ce qui vous obligera à utiliser vos mains pour escalader les parois rocheuses volcaniques et à vous frayer un chemin dans les sentiers parsemés de racines.
+La section de la "Tête de Lion" offre une véritable exposition, où l'on doit être très précis. Votre effort vous vaudra l'un des plus beaux panoramas de l'île Maurice : une vue à 360 degrés sur le lagon turquoise, la ceinture sucrière et le site de la bataille de Grand Port en 1810, la seule victoire navale des Français napoléoniens. En raison de la technicité de l'ascension et du risque élevé de glissade sur le sol argileux, ce sentier ne doit être emprunté que par temps sec et par des randonneurs expérimentés.</t>
+  </si>
+  <si>
+    <t>Sentier d'Alexandra Falls</t>
+  </si>
+  <si>
+    <t>2,7km 157mD+ 1h30.  Synthèse courte à faire : Partez découvrir cet itinéraire aller-retour de 2,7-km près de St. Martin, Savanne. Généralement considéré comme un parcours modéré, il faut en moyenne 1 h 2 min pour le parcourir. C’est un endroit très prisé pour l'ornithologie, la randonnée et le VTT, vous croiserez donc probablement du monde pendant votre excursion. La meilleure période de visite est de mars à janvier. Les chiens sont les bienvenus et peuvent être lâchés à certains endroits.</t>
+  </si>
+  <si>
+    <t>Parc national gorges rivière noire</t>
+  </si>
+  <si>
+    <t>6,9 km
+Distance
+456 m
+Dénivelé positif
+SYNTHESE BEAUCOUP PLUS COURTE A FAIRE:
+S'élevant de façon spectaculaire dans le lagon turquoise de l'océan Indien, ce monolithe basaltique emblématique offre l'une des aventures les plus importantes sur le plan culturel et les plus exigeantes sur le plan physique à l'île Maurice. Classé au patrimoine mondial de l'UNESCO, le Morne Brabant est imprégné de l'histoire tragique de la "République marron". Il a servi de refuge aux esclaves en fuite qui, selon la légende, ont préféré se jeter du haut des falaises plutôt que d'être repris.
+Le sentier se divise en deux parties. La première partie est une piste large et trompeuse qui serpente doucement à travers une forêt sèche, accessible à la plupart des personnes en bonne condition physique. Cependant, après le panneau d'avertissement sur le plateau, l'itinéraire se transforme en un véritable défi d'alpinisme. Les randonneurs doivent s'attaquer à une escalade technique, en se servant de leurs mains et de leurs pieds pour franchir des parois rocheuses abruptes et la fameuse brèche en "V". L'exposition est réelle et le basalte peut être glissant, il est donc essentiel d'être sûr de soi.
+Votre récompense à la croix du sommet (490 mètres) est un panorama sans pareil sur les récifs du sud-ouest et l'illusion de la fameuse "cascade sous-marine" au large de la côte. Bien que la randonnée indépendante soit autorisée, un guide est fortement recommandé pour l'ascension finale en raison de la nature technique de l'ascension. Commencez au lever du soleil pour éviter la chaleur tropicale et la foule sur les crêtes étroites.</t>
+  </si>
+  <si>
+    <t>2,3 km
+Distance
+116 m
+Dénivelé positif
+Boucle
+SYNTHSE BEACOUP PLUS COURTE DE: Voici une magnifique randonnée qui longe la rivière Tamarin et mène aux chutes de Tamarin (également connues sous le nom de chutes de Tamarind), une série de sept cascades sur le plateau central de l'île Maurice. Le sentier traverse une épaisse forêt verdoyante et offre des vues époustouflantes. À la bonne saison, il est possible de se baigner dans ce qui ressemble à un paradis. Les randonneurs recommandent d'apporter une serviette légère, de la crème solaire, un maillot de bain et de bonnes chaussures avec une bonne adhérence ou même des chaussures d'eau. Veuillez noter que le chemin près des chutes d'eau peut être très glissant. Certains passages peuvent nécessiter l'utilisation des mains pour garder l'équilibre et ce sentier ne doit pas être emprunté après la pluie.</t>
+  </si>
+  <si>
+    <t>Boucle courte des 7 cascades</t>
+  </si>
+  <si>
+    <t>4,3 km
+Distance
+370 m
+Dénivelé positif
+Aller-retour
+Ce sentier gratifiant vous emmène au sommet de la troisième plus haute montagne de l'île Maurice, Le Pouce (812 m), connu localement sous le nom de "The Thumb" (le pouce) en raison de son pinacle rocheux caractéristique. Il vous conduit à travers des champs de canne à sucre et des forêts tropicales luxuriantes avant d'atteindre les hauteurs rocheuses balayées par le vent.
+L'itinéraire le plus populaire et le plus accessible part du village de Petit Verger (près de Saint-Pierre) et suit un sentier clairement balisé qui traverse des champs de canne à sucre et des forêts avant de déboucher sur des pentes herbeuses. À l'approche du sommet, le terrain se transforme en une escalade raide et physique qui nécessite des chaussures solides et l'utilisation des mains pour naviguer sur la roche volcanique.
+Vous serez récompensé par une vue à 360 degrés sur la capitale Port Louis, la chaîne de Moka et les îles du nord comme Coin de Mire. Les randonneurs doivent être prêts à affronter la boue glissante, surtout après les fréquentes pluies de l'île, qui peuvent rendre le sentier dangereux.</t>
+  </si>
+  <si>
+    <t>5,8 km
+Distance
+327 m
+Dénivelé positif
+Boucle
+Embarquez pour une aventure palpitante le long de la rivière Tamarind, qui abrite les emblématiques 7 Cascades (Tamarind Falls). Cet itinéraire près d'Henrietta est moins une randonnée qu'une escalade dans le canyon ; le "sentier" est souvent une piste faible et boueuse qui vous oblige à vous accrocher aux racines des goyaviers et à naviguer sur des parois abruptes de basalte pour atteindre les bassins cachés.
+Vous descendrez profondément dans la gorge, en sautant sur les rochers de la rivière et en passant derrière des rideaux d'eau tonitruants. Le terrain est célèbre pour être glissant et escarpé, ce qui exige des chaussures à haute adhérence et souvent l'utilisation des mains (ou de cordes fixes) pour franchir les dénivelés en toute sécurité.
+Bien que la baignade dans les bassins frais et émeraude soit rafraîchissante, les visiteurs doivent être vigilants face aux crues soudaines et au réseau confus de sentiers informels. En raison de la nature technique de la descente et du manque de signalisation, il est fortement recommandé de faire appel à un guide local pour découvrir en toute sécurité la séquence complète de ces magnifiques chutes, dont la principale fait une chute de près de 300 mètres.</t>
+  </si>
+  <si>
+    <t>Boucle des cascades</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -22584,6 +22669,29 @@
       <sz val="10"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="24"/>
+      <color rgb="FF161F13"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF535B52"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF161F13"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -22610,7 +22718,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -22619,6 +22727,25 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -26414,7 +26541,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -26450,7 +26577,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="409.6" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>1185</v>
       </c>
@@ -26459,7 +26586,9 @@
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
+      <c r="E4" s="8" t="s">
+        <v>7485</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
@@ -26487,7 +26616,7 @@
       </c>
       <c r="E6" s="5"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="328.5" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>1193</v>
       </c>
@@ -26496,7 +26625,9 @@
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
+      <c r="E7" s="8" t="s">
+        <v>7481</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
@@ -26509,7 +26640,7 @@
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="409.6" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>1197</v>
       </c>
@@ -26518,7 +26649,9 @@
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+      <c r="E9" s="13" t="s">
+        <v>7488</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
@@ -26872,7 +27005,44 @@
       <c r="D37" s="5"/>
       <c r="E37" s="5"/>
     </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
+        <v>7482</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>7484</v>
+      </c>
+      <c r="E38" t="s">
+        <v>7483</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="315" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
+        <v>7487</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>7486</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A40" s="14" t="s">
+        <v>7490</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>7489</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="E41" s="10"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E42" s="11"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E43" s="12"/>
+    </row>
   </sheetData>
+  <autoFilter ref="A3:E3" xr:uid="{00000000-0001-0000-1200-000000000000}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -26882,6 +27052,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr>
+    <tabColor theme="6" tint="0.59999389629810485"/>
+  </sheetPr>
   <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -31358,13 +31531,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr>
+    <tabColor theme="6" tint="0.59999389629810485"/>
+  </sheetPr>
   <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="4" max="4" width="28" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="50" customWidth="1"/>
   </cols>
   <sheetData>
@@ -31448,7 +31624,9 @@
       <c r="D7" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="E7" s="5"/>
+      <c r="E7" s="5" t="s">
+        <v>7473</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
@@ -31491,7 +31669,9 @@
       <c r="D10" s="5" t="s">
         <v>272</v>
       </c>
-      <c r="E10" s="5"/>
+      <c r="E10" s="5" t="s">
+        <v>7474</v>
+      </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
@@ -31506,7 +31686,9 @@
       <c r="D11" s="5" t="s">
         <v>276</v>
       </c>
-      <c r="E11" s="5"/>
+      <c r="E11" s="5" t="s">
+        <v>7475</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
@@ -31536,7 +31718,9 @@
       <c r="D13" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="E13" s="5"/>
+      <c r="E13" s="5" t="s">
+        <v>7474</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
@@ -31551,7 +31735,9 @@
       <c r="D14" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="E14" s="5"/>
+      <c r="E14" s="5" t="s">
+        <v>7474</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
@@ -31564,7 +31750,9 @@
         <v>291</v>
       </c>
       <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
+      <c r="E15" s="5" t="s">
+        <v>7475</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
@@ -31579,7 +31767,9 @@
       <c r="D16" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="E16" s="5"/>
+      <c r="E16" s="5" t="s">
+        <v>7473</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -35369,13 +35559,16 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr filterMode="1">
+    <tabColor theme="6" tint="0.59999389629810485"/>
+  </sheetPr>
   <dimension ref="A1:E179"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="4" max="4" width="28" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="50" customWidth="1"/>
   </cols>
   <sheetData>
@@ -35405,7 +35598,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>294</v>
       </c>
@@ -35480,7 +35673,7 @@
       </c>
       <c r="E8" s="5"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>314</v>
       </c>
@@ -35493,7 +35686,9 @@
       <c r="D9" s="5" t="s">
         <v>317</v>
       </c>
-      <c r="E9" s="5"/>
+      <c r="E9" s="5" t="s">
+        <v>7478</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
@@ -35508,9 +35703,11 @@
       <c r="D10" s="5" t="s">
         <v>321</v>
       </c>
-      <c r="E10" s="5"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E10" s="5" t="s">
+        <v>7480</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>322</v>
       </c>
@@ -35523,9 +35720,11 @@
       <c r="D11" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="E11" s="5"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E11" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>326</v>
       </c>
@@ -35538,9 +35737,11 @@
       <c r="D12" s="5" t="s">
         <v>329</v>
       </c>
-      <c r="E12" s="5"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E12" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>330</v>
       </c>
@@ -35555,7 +35756,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>334</v>
       </c>
@@ -35568,7 +35769,9 @@
       <c r="D14" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="E14" s="5"/>
+      <c r="E14" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
@@ -35683,7 +35886,7 @@
       <c r="D23" s="5"/>
       <c r="E23" s="5"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>362</v>
       </c>
@@ -35696,7 +35899,9 @@
       <c r="D24" s="5" t="s">
         <v>365</v>
       </c>
-      <c r="E24" s="5"/>
+      <c r="E24" s="5" t="s">
+        <v>7478</v>
+      </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
@@ -35711,7 +35916,7 @@
       <c r="D25" s="5"/>
       <c r="E25" s="5"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>369</v>
       </c>
@@ -35722,9 +35927,11 @@
         <v>371</v>
       </c>
       <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E26" s="5" t="s">
+        <v>7476</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>372</v>
       </c>
@@ -35733,7 +35940,9 @@
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
+      <c r="E27" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
@@ -35748,7 +35957,7 @@
       <c r="D28" s="5"/>
       <c r="E28" s="5"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>377</v>
       </c>
@@ -35759,9 +35968,11 @@
         <v>379</v>
       </c>
       <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E29" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>380</v>
       </c>
@@ -35774,9 +35985,11 @@
       <c r="D30" s="5" t="s">
         <v>383</v>
       </c>
-      <c r="E30" s="5"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E30" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>384</v>
       </c>
@@ -35789,9 +36002,11 @@
       <c r="D31" s="5" t="s">
         <v>387</v>
       </c>
-      <c r="E31" s="5"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E31" s="5" t="s">
+        <v>7477</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>388</v>
       </c>
@@ -35804,9 +36019,11 @@
       <c r="D32" s="5" t="s">
         <v>390</v>
       </c>
-      <c r="E32" s="5"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E32" s="5" t="s">
+        <v>7478</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>391</v>
       </c>
@@ -35819,9 +36036,11 @@
       <c r="D33" s="5" t="s">
         <v>313</v>
       </c>
-      <c r="E33" s="5"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E33" s="5" t="s">
+        <v>7478</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>392</v>
       </c>
@@ -35832,9 +36051,11 @@
         <v>394</v>
       </c>
       <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E34" s="5" t="s">
+        <v>7478</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>395</v>
       </c>
@@ -35845,7 +36066,9 @@
         <v>397</v>
       </c>
       <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
+      <c r="E35" s="5" t="s">
+        <v>7478</v>
+      </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
@@ -35858,7 +36081,7 @@
       <c r="D36" s="5"/>
       <c r="E36" s="5"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
         <v>400</v>
       </c>
@@ -35869,9 +36092,11 @@
         <v>402</v>
       </c>
       <c r="D37" s="5"/>
-      <c r="E37" s="5"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E37" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
         <v>403</v>
       </c>
@@ -35884,9 +36109,11 @@
       <c r="D38" s="5" t="s">
         <v>406</v>
       </c>
-      <c r="E38" s="5"/>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E38" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>407</v>
       </c>
@@ -35899,7 +36126,9 @@
       <c r="D39" s="5" t="s">
         <v>410</v>
       </c>
-      <c r="E39" s="5"/>
+      <c r="E39" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
@@ -35914,7 +36143,7 @@
       <c r="D40" s="5"/>
       <c r="E40" s="5"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
         <v>414</v>
       </c>
@@ -35927,9 +36156,11 @@
       <c r="D41" s="5" t="s">
         <v>417</v>
       </c>
-      <c r="E41" s="5"/>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E41" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>418</v>
       </c>
@@ -35942,9 +36173,11 @@
       <c r="D42" s="5" t="s">
         <v>421</v>
       </c>
-      <c r="E42" s="5"/>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E42" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
         <v>422</v>
       </c>
@@ -35957,9 +36190,11 @@
       <c r="D43" s="5" t="s">
         <v>425</v>
       </c>
-      <c r="E43" s="5"/>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E43" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>426</v>
       </c>
@@ -35970,9 +36205,11 @@
         <v>428</v>
       </c>
       <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E44" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>429</v>
       </c>
@@ -35983,7 +36220,9 @@
         <v>431</v>
       </c>
       <c r="D45" s="5"/>
-      <c r="E45" s="5"/>
+      <c r="E45" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
@@ -36000,7 +36239,7 @@
       </c>
       <c r="E46" s="5"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>436</v>
       </c>
@@ -36011,9 +36250,11 @@
         <v>438</v>
       </c>
       <c r="D47" s="5"/>
-      <c r="E47" s="5"/>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E47" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
         <v>439</v>
       </c>
@@ -36024,9 +36265,11 @@
         <v>441</v>
       </c>
       <c r="D48" s="5"/>
-      <c r="E48" s="5"/>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E48" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
         <v>442</v>
       </c>
@@ -36037,9 +36280,11 @@
         <v>444</v>
       </c>
       <c r="D49" s="5"/>
-      <c r="E49" s="5"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E49" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
         <v>445</v>
       </c>
@@ -36050,9 +36295,11 @@
         <v>447</v>
       </c>
       <c r="D50" s="5"/>
-      <c r="E50" s="5"/>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E50" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
         <v>448</v>
       </c>
@@ -36065,9 +36312,11 @@
       <c r="D51" s="5" t="s">
         <v>451</v>
       </c>
-      <c r="E51" s="5"/>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E51" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
         <v>452</v>
       </c>
@@ -36078,9 +36327,11 @@
         <v>454</v>
       </c>
       <c r="D52" s="5"/>
-      <c r="E52" s="5"/>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E52" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
         <v>455</v>
       </c>
@@ -36093,9 +36344,11 @@
       <c r="D53" s="5" t="s">
         <v>313</v>
       </c>
-      <c r="E53" s="5"/>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E53" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
         <v>458</v>
       </c>
@@ -36106,7 +36359,9 @@
         <v>460</v>
       </c>
       <c r="D54" s="5"/>
-      <c r="E54" s="5"/>
+      <c r="E54" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
@@ -36138,7 +36393,7 @@
       </c>
       <c r="E56" s="5"/>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
         <v>468</v>
       </c>
@@ -36149,7 +36404,9 @@
         <v>470</v>
       </c>
       <c r="D57" s="5"/>
-      <c r="E57" s="5"/>
+      <c r="E57" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
@@ -36166,7 +36423,7 @@
       </c>
       <c r="E58" s="5"/>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
         <v>475</v>
       </c>
@@ -36177,9 +36434,11 @@
         <v>477</v>
       </c>
       <c r="D59" s="5"/>
-      <c r="E59" s="5"/>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E59" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
         <v>478</v>
       </c>
@@ -36192,9 +36451,11 @@
       <c r="D60" s="5" t="s">
         <v>481</v>
       </c>
-      <c r="E60" s="5"/>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E60" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
         <v>482</v>
       </c>
@@ -36205,9 +36466,11 @@
         <v>484</v>
       </c>
       <c r="D61" s="5"/>
-      <c r="E61" s="5"/>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E61" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
         <v>485</v>
       </c>
@@ -36218,9 +36481,11 @@
         <v>487</v>
       </c>
       <c r="D62" s="5"/>
-      <c r="E62" s="5"/>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E62" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
         <v>488</v>
       </c>
@@ -36231,9 +36496,11 @@
         <v>490</v>
       </c>
       <c r="D63" s="5"/>
-      <c r="E63" s="5"/>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E63" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
         <v>491</v>
       </c>
@@ -36244,7 +36511,9 @@
         <v>493</v>
       </c>
       <c r="D64" s="5"/>
-      <c r="E64" s="5"/>
+      <c r="E64" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
@@ -36259,7 +36528,7 @@
       <c r="D65" s="5"/>
       <c r="E65" s="5"/>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
         <v>497</v>
       </c>
@@ -36270,9 +36539,11 @@
         <v>499</v>
       </c>
       <c r="D66" s="5"/>
-      <c r="E66" s="5"/>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E66" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
         <v>500</v>
       </c>
@@ -36283,9 +36554,11 @@
         <v>502</v>
       </c>
       <c r="D67" s="5"/>
-      <c r="E67" s="5"/>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E67" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
         <v>503</v>
       </c>
@@ -36294,7 +36567,9 @@
       </c>
       <c r="C68" s="5"/>
       <c r="D68" s="5"/>
-      <c r="E68" s="5"/>
+      <c r="E68" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
@@ -36309,7 +36584,7 @@
       <c r="D69" s="5"/>
       <c r="E69" s="5"/>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
         <v>508</v>
       </c>
@@ -36320,7 +36595,9 @@
         <v>493</v>
       </c>
       <c r="D70" s="5"/>
-      <c r="E70" s="5"/>
+      <c r="E70" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
@@ -36337,7 +36614,7 @@
       </c>
       <c r="E71" s="5"/>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
         <v>514</v>
       </c>
@@ -36350,9 +36627,11 @@
       <c r="D72" s="5" t="s">
         <v>517</v>
       </c>
-      <c r="E72" s="5"/>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E72" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
         <v>518</v>
       </c>
@@ -36363,9 +36642,11 @@
         <v>520</v>
       </c>
       <c r="D73" s="5"/>
-      <c r="E73" s="5"/>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E73" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
         <v>521</v>
       </c>
@@ -36376,9 +36657,11 @@
       <c r="D74" s="5" t="s">
         <v>523</v>
       </c>
-      <c r="E74" s="5"/>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E74" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="5" t="s">
         <v>524</v>
       </c>
@@ -36389,9 +36672,11 @@
         <v>526</v>
       </c>
       <c r="D75" s="5"/>
-      <c r="E75" s="5"/>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E75" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="s">
         <v>527</v>
       </c>
@@ -36400,7 +36685,9 @@
       </c>
       <c r="C76" s="5"/>
       <c r="D76" s="5"/>
-      <c r="E76" s="5"/>
+      <c r="E76" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
@@ -36437,7 +36724,7 @@
       <c r="D79" s="5"/>
       <c r="E79" s="5"/>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
         <v>536</v>
       </c>
@@ -36446,9 +36733,11 @@
       </c>
       <c r="C80" s="5"/>
       <c r="D80" s="5"/>
-      <c r="E80" s="5"/>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E80" s="5" t="s">
+        <v>7478</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
         <v>538</v>
       </c>
@@ -36459,9 +36748,11 @@
         <v>540</v>
       </c>
       <c r="D81" s="5"/>
-      <c r="E81" s="5"/>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E81" s="5" t="s">
+        <v>7478</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
         <v>541</v>
       </c>
@@ -36474,9 +36765,11 @@
       <c r="D82" s="5" t="s">
         <v>544</v>
       </c>
-      <c r="E82" s="5"/>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E82" s="5" t="s">
+        <v>7478</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
         <v>545</v>
       </c>
@@ -36485,9 +36778,11 @@
       </c>
       <c r="C83" s="5"/>
       <c r="D83" s="5"/>
-      <c r="E83" s="5"/>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E83" s="5" t="s">
+        <v>7478</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="5" t="s">
         <v>547</v>
       </c>
@@ -36498,9 +36793,11 @@
         <v>549</v>
       </c>
       <c r="D84" s="5"/>
-      <c r="E84" s="5"/>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E84" s="5" t="s">
+        <v>7478</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="5" t="s">
         <v>550</v>
       </c>
@@ -36511,7 +36808,9 @@
         <v>552</v>
       </c>
       <c r="D85" s="5"/>
-      <c r="E85" s="5"/>
+      <c r="E85" s="5" t="s">
+        <v>7478</v>
+      </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
@@ -36580,7 +36879,7 @@
       <c r="D90" s="5"/>
       <c r="E90" s="5"/>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="5" t="s">
         <v>568</v>
       </c>
@@ -36593,9 +36892,11 @@
       <c r="D91" s="5" t="s">
         <v>571</v>
       </c>
-      <c r="E91" s="5"/>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E91" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="5" t="s">
         <v>572</v>
       </c>
@@ -36604,9 +36905,11 @@
       </c>
       <c r="C92" s="5"/>
       <c r="D92" s="5"/>
-      <c r="E92" s="5"/>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E92" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="5" t="s">
         <v>574</v>
       </c>
@@ -36617,9 +36920,11 @@
         <v>576</v>
       </c>
       <c r="D93" s="5"/>
-      <c r="E93" s="5"/>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E93" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="5" t="s">
         <v>577</v>
       </c>
@@ -36628,9 +36933,11 @@
       </c>
       <c r="C94" s="5"/>
       <c r="D94" s="5"/>
-      <c r="E94" s="5"/>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E94" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="5" t="s">
         <v>579</v>
       </c>
@@ -36641,9 +36948,11 @@
         <v>581</v>
       </c>
       <c r="D95" s="5"/>
-      <c r="E95" s="5"/>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E95" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="5" t="s">
         <v>582</v>
       </c>
@@ -36654,9 +36963,11 @@
         <v>584</v>
       </c>
       <c r="D96" s="5"/>
-      <c r="E96" s="5"/>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E96" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="5" t="s">
         <v>585</v>
       </c>
@@ -36667,9 +36978,11 @@
       <c r="D97" s="5" t="s">
         <v>587</v>
       </c>
-      <c r="E97" s="5"/>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E97" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="5" t="s">
         <v>588</v>
       </c>
@@ -36682,9 +36995,11 @@
       <c r="D98" s="5" t="s">
         <v>591</v>
       </c>
-      <c r="E98" s="5"/>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E98" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="5" t="s">
         <v>592</v>
       </c>
@@ -36697,9 +37012,11 @@
       <c r="D99" s="5" t="s">
         <v>595</v>
       </c>
-      <c r="E99" s="5"/>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E99" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="5" t="s">
         <v>596</v>
       </c>
@@ -36712,9 +37029,11 @@
       <c r="D100" s="5" t="s">
         <v>599</v>
       </c>
-      <c r="E100" s="5"/>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E100" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="5" t="s">
         <v>600</v>
       </c>
@@ -36725,9 +37044,11 @@
         <v>602</v>
       </c>
       <c r="D101" s="5"/>
-      <c r="E101" s="5"/>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E101" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="5" t="s">
         <v>603</v>
       </c>
@@ -36738,9 +37059,11 @@
         <v>605</v>
       </c>
       <c r="D102" s="5"/>
-      <c r="E102" s="5"/>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E102" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="5" t="s">
         <v>606</v>
       </c>
@@ -36753,9 +37076,11 @@
       <c r="D103" s="5" t="s">
         <v>609</v>
       </c>
-      <c r="E103" s="5"/>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E103" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="5" t="s">
         <v>610</v>
       </c>
@@ -36766,9 +37091,11 @@
         <v>612</v>
       </c>
       <c r="D104" s="5"/>
-      <c r="E104" s="5"/>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E104" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="5" t="s">
         <v>613</v>
       </c>
@@ -36777,7 +37104,9 @@
       </c>
       <c r="C105" s="5"/>
       <c r="D105" s="5"/>
-      <c r="E105" s="5"/>
+      <c r="E105" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="5" t="s">
@@ -36824,7 +37153,7 @@
       </c>
       <c r="E108" s="5"/>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="5" t="s">
         <v>627</v>
       </c>
@@ -36835,7 +37164,9 @@
         <v>629</v>
       </c>
       <c r="D109" s="5"/>
-      <c r="E109" s="5"/>
+      <c r="E109" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="5" t="s">
@@ -36923,7 +37254,7 @@
       </c>
       <c r="E115" s="5"/>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" s="5" t="s">
         <v>651</v>
       </c>
@@ -36934,9 +37265,11 @@
         <v>653</v>
       </c>
       <c r="D116" s="5"/>
-      <c r="E116" s="5"/>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E116" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="5" t="s">
         <v>654</v>
       </c>
@@ -36947,9 +37280,11 @@
         <v>656</v>
       </c>
       <c r="D117" s="5"/>
-      <c r="E117" s="5"/>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E117" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="5" t="s">
         <v>657</v>
       </c>
@@ -36962,9 +37297,11 @@
       <c r="D118" s="5" t="s">
         <v>660</v>
       </c>
-      <c r="E118" s="5"/>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E118" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="5" t="s">
         <v>661</v>
       </c>
@@ -36975,9 +37312,11 @@
         <v>663</v>
       </c>
       <c r="D119" s="5"/>
-      <c r="E119" s="5"/>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E119" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="5" t="s">
         <v>664</v>
       </c>
@@ -36990,9 +37329,11 @@
       <c r="D120" s="5" t="s">
         <v>667</v>
       </c>
-      <c r="E120" s="5"/>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E120" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="5" t="s">
         <v>668</v>
       </c>
@@ -37003,9 +37344,11 @@
         <v>670</v>
       </c>
       <c r="D121" s="5"/>
-      <c r="E121" s="5"/>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E121" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" s="5" t="s">
         <v>671</v>
       </c>
@@ -37014,9 +37357,11 @@
       </c>
       <c r="C122" s="5"/>
       <c r="D122" s="5"/>
-      <c r="E122" s="5"/>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E122" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="5" t="s">
         <v>673</v>
       </c>
@@ -37027,9 +37372,11 @@
         <v>675</v>
       </c>
       <c r="D123" s="5"/>
-      <c r="E123" s="5"/>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E123" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" s="5" t="s">
         <v>676</v>
       </c>
@@ -37042,9 +37389,11 @@
       <c r="D124" s="5" t="s">
         <v>679</v>
       </c>
-      <c r="E124" s="5"/>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E124" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" s="5" t="s">
         <v>680</v>
       </c>
@@ -37055,9 +37404,11 @@
         <v>682</v>
       </c>
       <c r="D125" s="5"/>
-      <c r="E125" s="5"/>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E125" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" s="5" t="s">
         <v>683</v>
       </c>
@@ -37068,9 +37419,11 @@
         <v>685</v>
       </c>
       <c r="D126" s="5"/>
-      <c r="E126" s="5"/>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E126" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" s="5" t="s">
         <v>686</v>
       </c>
@@ -37081,7 +37434,9 @@
         <v>688</v>
       </c>
       <c r="D127" s="5"/>
-      <c r="E127" s="5"/>
+      <c r="E127" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="5" t="s">
@@ -37098,7 +37453,7 @@
       </c>
       <c r="E128" s="5"/>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" s="5" t="s">
         <v>692</v>
       </c>
@@ -37109,7 +37464,9 @@
         <v>694</v>
       </c>
       <c r="D129" s="5"/>
-      <c r="E129" s="5"/>
+      <c r="E129" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="5" t="s">
@@ -37124,7 +37481,7 @@
       <c r="D130" s="5"/>
       <c r="E130" s="5"/>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="5" t="s">
         <v>697</v>
       </c>
@@ -37133,7 +37490,9 @@
       </c>
       <c r="C131" s="5"/>
       <c r="D131" s="5"/>
-      <c r="E131" s="5"/>
+      <c r="E131" s="5" t="s">
+        <v>7478</v>
+      </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="5" t="s">
@@ -37200,7 +37559,7 @@
       </c>
       <c r="E136" s="5"/>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" s="5" t="s">
         <v>714</v>
       </c>
@@ -37211,9 +37570,11 @@
         <v>716</v>
       </c>
       <c r="D137" s="5"/>
-      <c r="E137" s="5"/>
-    </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E137" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" s="5" t="s">
         <v>717</v>
       </c>
@@ -37224,9 +37585,11 @@
         <v>719</v>
       </c>
       <c r="D138" s="5"/>
-      <c r="E138" s="5"/>
-    </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E138" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="5" t="s">
         <v>720</v>
       </c>
@@ -37237,7 +37600,9 @@
         <v>722</v>
       </c>
       <c r="D139" s="5"/>
-      <c r="E139" s="5"/>
+      <c r="E139" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="5" t="s">
@@ -37254,7 +37619,7 @@
       </c>
       <c r="E140" s="5"/>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" s="5" t="s">
         <v>727</v>
       </c>
@@ -37265,7 +37630,9 @@
         <v>729</v>
       </c>
       <c r="D141" s="5"/>
-      <c r="E141" s="5"/>
+      <c r="E141" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="5" t="s">
@@ -37289,7 +37656,7 @@
       <c r="D143" s="5"/>
       <c r="E143" s="5"/>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" s="5" t="s">
         <v>734</v>
       </c>
@@ -37300,7 +37667,9 @@
         <v>736</v>
       </c>
       <c r="D144" s="5"/>
-      <c r="E144" s="5"/>
+      <c r="E144" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="5" t="s">
@@ -37315,7 +37684,7 @@
       <c r="D145" s="5"/>
       <c r="E145" s="5"/>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" s="5" t="s">
         <v>740</v>
       </c>
@@ -37326,7 +37695,9 @@
         <v>742</v>
       </c>
       <c r="D146" s="5"/>
-      <c r="E146" s="5"/>
+      <c r="E146" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="5" t="s">
@@ -37339,7 +37710,7 @@
       <c r="D147" s="5"/>
       <c r="E147" s="5"/>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" s="5" t="s">
         <v>745</v>
       </c>
@@ -37350,7 +37721,9 @@
         <v>747</v>
       </c>
       <c r="D148" s="5"/>
-      <c r="E148" s="5"/>
+      <c r="E148" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="5" t="s">
@@ -37365,7 +37738,7 @@
       <c r="D149" s="5"/>
       <c r="E149" s="5"/>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" s="5" t="s">
         <v>751</v>
       </c>
@@ -37376,7 +37749,9 @@
         <v>753</v>
       </c>
       <c r="D150" s="5"/>
-      <c r="E150" s="5"/>
+      <c r="E150" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="5" t="s">
@@ -37391,7 +37766,7 @@
       <c r="D151" s="5"/>
       <c r="E151" s="5"/>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" s="5" t="s">
         <v>757</v>
       </c>
@@ -37402,7 +37777,9 @@
         <v>759</v>
       </c>
       <c r="D152" s="5"/>
-      <c r="E152" s="5"/>
+      <c r="E152" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="5" t="s">
@@ -37430,7 +37807,7 @@
       <c r="D154" s="5"/>
       <c r="E154" s="5"/>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" s="5" t="s">
         <v>766</v>
       </c>
@@ -37441,7 +37818,9 @@
         <v>768</v>
       </c>
       <c r="D155" s="5"/>
-      <c r="E155" s="5"/>
+      <c r="E155" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="5" t="s">
@@ -37458,7 +37837,7 @@
       </c>
       <c r="E156" s="5"/>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="5" t="s">
         <v>773</v>
       </c>
@@ -37467,9 +37846,11 @@
       </c>
       <c r="C157" s="5"/>
       <c r="D157" s="5"/>
-      <c r="E157" s="5"/>
-    </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E157" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" s="5" t="s">
         <v>775</v>
       </c>
@@ -37480,7 +37861,9 @@
         <v>777</v>
       </c>
       <c r="D158" s="5"/>
-      <c r="E158" s="5"/>
+      <c r="E158" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="5" t="s">
@@ -37497,7 +37880,7 @@
       </c>
       <c r="E159" s="5"/>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" s="5" t="s">
         <v>782</v>
       </c>
@@ -37510,7 +37893,9 @@
       <c r="D160" s="5" t="s">
         <v>785</v>
       </c>
-      <c r="E160" s="5"/>
+      <c r="E160" s="5" t="s">
+        <v>7479</v>
+      </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="5" t="s">
@@ -37536,7 +37921,7 @@
       <c r="D162" s="5"/>
       <c r="E162" s="5"/>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" s="5" t="s">
         <v>791</v>
       </c>
@@ -37549,9 +37934,11 @@
       <c r="D163" s="5" t="s">
         <v>794</v>
       </c>
-      <c r="E163" s="5"/>
-    </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E163" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" s="5" t="s">
         <v>795</v>
       </c>
@@ -37562,9 +37949,11 @@
         <v>797</v>
       </c>
       <c r="D164" s="5"/>
-      <c r="E164" s="5"/>
-    </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E164" s="5" t="s">
+        <v>7479</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" s="5" t="s">
         <v>798</v>
       </c>
@@ -37577,9 +37966,11 @@
       <c r="D165" s="5" t="s">
         <v>801</v>
       </c>
-      <c r="E165" s="5"/>
-    </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E165" s="5" t="s">
+        <v>7478</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" s="5" t="s">
         <v>802</v>
       </c>
@@ -37590,7 +37981,9 @@
         <v>804</v>
       </c>
       <c r="D166" s="5"/>
-      <c r="E166" s="5"/>
+      <c r="E166" s="5" t="s">
+        <v>7478</v>
+      </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="5" t="s">
@@ -37762,6 +38155,11 @@
       <c r="E179" s="5"/>
     </row>
   </sheetData>
+  <autoFilter ref="A3:E179" xr:uid="{00000000-0001-0000-0300-000000000000}">
+    <filterColumn colId="4">
+      <filters blank="1"/>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>

</xml_diff>